<commit_message>
BRD-04 Collections screenshots retaken in the BDO style-guide presentation on a fresh seed stack: 102 images; FRS, guide deck, sign-off workbook and UX documents 07 to 09 rebuilt at v2.0; capture widens the window for a list that scrolls sideways in its card and grows it to show a dialog taller than the window
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Drop-1_Transactional/BRD-04_Collections/03_BIBS_Signoff_BRD-04_Collections_v2.0.xlsx
+++ b/docs/deliverables/out/Drop-1_Transactional/BRD-04_Collections/03_BIBS_Signoff_BRD-04_Collections_v2.0.xlsx
@@ -35365,7 +35365,7 @@
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
-          <t>Lists show status tabs, a search box, a Filters button for the other criteria and the paged table ("Showing 1 to n of N results"). A row opens its record. Dates show as dd-MMM-yyyy and times as dd-MMM-yyyy HH:mm in Philippine time. Selecting rows enables the actions of the tab, which apply to every selected row.</t>
+          <t>Lists show status tabs, a search box, a Filters button for the other criteria and the paged table ("Showing 1 to n of N results"). Rows alternate white and Background Blue; a long list scrolls inside its card with the header row in view. A row opens its record. Dates show as dd-MMM-yyyy and times as dd-MMM-yyyy HH:mm in Philippine time. Selecting rows enables the actions of the tab, which apply to every selected row.</t>
         </is>
       </c>
       <c r="D7" s="12" t="n"/>
@@ -35479,7 +35479,7 @@
       </c>
       <c r="C13" s="12" t="inlineStr">
         <is>
-          <t>Statuses are pills of one size and colour per state group; a pill never wraps. Statuses show their full label; an agreed short form, with the full label in the tooltip, is used only for a label longer than 21 characters. Dispositions are tags with the category under them.</t>
+          <t>Statuses are outlined pills of one size and colour per state group; a pill never wraps. Statuses show their full label; an agreed short form, with the full label in the tooltip, is used only for a label longer than 21 characters. Dispositions are tags with the category under them.</t>
         </is>
       </c>
       <c r="D13" s="12" t="n"/>

</xml_diff>